<commit_message>
Stage 8 review fixes: C-020
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/KT12/MV-2021-284/MV-2021-284_AssayWorksheet_122021_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/KT12/MV-2021-284/MV-2021-284_AssayWorksheet_122021_v03.xlsx
@@ -164,7 +164,7 @@
   <commentList>
     <comment ref="A3" authorId="0" shapeId="0">
       <text>
-        <t>Check the donor pool lots against the receipt sheet before this is filed</t>
+        <t>Use the receipt records for donor-pool and matrix-lot identities.</t>
       </text>
     </comment>
   </commentList>
@@ -179,7 +179,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>See the readout for the clearance route discussion. Do not quote these values without the matrix acceptance sheet.</t>
+        <t>See the paired readout for the clearance-route discussion and the study records for matrix acceptance. Retain the per-million-cells units when quoting hepatocyte CLint.</t>
       </text>
     </comment>
   </commentList>
@@ -547,7 +547,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MV-2021-284 assay worksheet</t>
+          <t>Merrivoss Bioanalysis Inc, a Tarnovell company | MV-2021-284 assay worksheet</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>QC'd 12/20/2021</t>
+          <t>12/20/2021</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -700,14 +700,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Accession-lot mapping</t>
+          <t>Accession and matrix source records</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Accession lot</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -717,133 +717,49 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Lot description</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Storage</t>
+          <t>Source to consult</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M21/BIO/06539-01</t>
+          <t>M21/BIO/06539</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pooled human liver microsomes</t>
+          <t>Human and rat liver microsomes</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Human arm, microsomal screen</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>11/16/2021</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>-80 °C</t>
+          <t>Receipt and matrix-lot records linked to the study accession</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>M21/BIO/06539-02</t>
+          <t>M21/BIO/06539</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pooled rat liver microsomes</t>
+          <t>Cryopreserved human and rat hepatocytes</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Rat arm, microsomal screen</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>11/16/2021</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>-80 °C</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>M21/BIO/06539-03</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Cryopreserved human hepatocytes</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Human arm, hepatocyte screen</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>11/16/2021</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Liquid nitrogen vapour</t>
-        </is>
-      </c>
-    </row>
+          <t>Receipt and matrix-lot records linked to the study accession</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>M21/BIO/06539-04</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Cryopreserved rat hepatocytes</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Rat arm, hepatocyte screen</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>11/16/2021</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Liquid nitrogen vapour</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Lot numbers follow the project LIMS reference. Matrix lots are not reused across projects.</t>
+          <t>Individual matrix lots and storage history are recorded in the receipt records; the study accession is not a matrix-lot identifier.</t>
         </is>
       </c>
     </row>
@@ -880,7 +796,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>0.5 mg/mL protein, 1 µM. Runs passed matrix acceptance before release.</t>
+          <t>0.5 mg/mL protein, 1 µM. Human and rat CLint are reported per mg microsomal protein; matrix acceptance documentation is retained in the study records.</t>
         </is>
       </c>
     </row>

</xml_diff>